<commit_message>
fix(games): fill in the missing size for VALORANT
- games/VALORANT.jpg: sizeGB 0 -> 36.5
- +0 items, -0 items, 1 modified
- +0 images
- regenerated data.json from source.xlsx
</commit_message>
<xml_diff>
--- a/source.xlsx
+++ b/source.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bo2lz\Desktop\Drive Deals V1.0\Drive Deals V1.0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bo2lz\Desktop\Drive Deals V1.0\Drive Deals V1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FEC9187-E962-4E69-8641-31107AB20450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64C9AD2D-08AC-451B-B47D-913E0C09E34C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39114,7 +39114,7 @@
         <v>3198</v>
       </c>
       <c r="C1073">
-        <v>0</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="1074" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>